<commit_message>
Missed changes in dupes accruals
</commit_message>
<xml_diff>
--- a/data/stx_xlsx/REJLb.ST.xlsx
+++ b/data/stx_xlsx/REJLb.ST.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="414">
   <si>
     <t>Company Fundamentals - Income Statement</t>
   </si>
@@ -826,6 +826,9 @@
   </si>
   <si>
     <t>Liabilities to credit institutions (Do not use)</t>
+  </si>
+  <si>
+    <t>Convertible debentures (Do not use)</t>
   </si>
   <si>
     <t>Total non-current liabilities</t>
@@ -13873,8 +13876,8 @@
       <c r="W103" s="18"/>
     </row>
     <row r="104" ht="15.0" customHeight="1">
-      <c r="A104" s="14" t="s">
-        <v>252</v>
+      <c r="A104" s="26" t="s">
+        <v>269</v>
       </c>
       <c r="B104" s="18"/>
       <c r="C104" s="18"/>
@@ -13911,7 +13914,7 @@
     </row>
     <row r="105" ht="15.0" customHeight="1">
       <c r="A105" s="16" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B105" s="17">
         <v>435.86</v>
@@ -13982,7 +13985,7 @@
     </row>
     <row r="106" ht="15.0" customHeight="1">
       <c r="A106" s="16" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B106" s="17">
         <v>2046.75</v>
@@ -14053,7 +14056,7 @@
     </row>
     <row r="107" ht="15.0" customHeight="1">
       <c r="A107" s="14" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B107" s="19">
         <v>49.42</v>
@@ -14120,7 +14123,7 @@
     </row>
     <row r="108" ht="15.0" customHeight="1">
       <c r="A108" s="14" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B108" s="19">
         <v>40.13</v>
@@ -14187,7 +14190,7 @@
     </row>
     <row r="109" ht="15.0" customHeight="1">
       <c r="A109" s="14" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B109" s="18"/>
       <c r="C109" s="19">
@@ -14218,7 +14221,7 @@
     </row>
     <row r="110" ht="15.0" customHeight="1">
       <c r="A110" s="14" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B110" s="18"/>
       <c r="C110" s="19">
@@ -14249,7 +14252,7 @@
     </row>
     <row r="111" ht="15.0" customHeight="1">
       <c r="A111" s="14" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B111" s="15">
         <v>997.02</v>
@@ -14316,7 +14319,7 @@
     </row>
     <row r="112" ht="15.0" customHeight="1">
       <c r="A112" s="14" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B112" s="15">
         <v>1205.11</v>
@@ -14383,7 +14386,7 @@
     </row>
     <row r="113" ht="15.0" customHeight="1">
       <c r="A113" s="16" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B113" s="17">
         <v>2291.69</v>
@@ -14454,7 +14457,7 @@
     </row>
     <row r="114" ht="15.0" customHeight="1">
       <c r="A114" s="14" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B114" s="18">
         <v>0.0</v>
@@ -14509,7 +14512,7 @@
     </row>
     <row r="115" ht="15.0" customHeight="1">
       <c r="A115" s="16" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B115" s="20">
         <v>0.0</v>
@@ -14564,7 +14567,7 @@
     </row>
     <row r="116" ht="15.0" customHeight="1">
       <c r="A116" s="16" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B116" s="17">
         <v>2291.69</v>
@@ -14635,7 +14638,7 @@
     </row>
     <row r="117" ht="15.0" customHeight="1">
       <c r="A117" s="16" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B117" s="17">
         <v>4338.44</v>
@@ -14706,7 +14709,7 @@
     </row>
     <row r="118" ht="15.0" customHeight="1">
       <c r="A118" s="14" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B118" s="19">
         <v>22.58</v>
@@ -14777,7 +14780,7 @@
     </row>
     <row r="119" ht="15.0" customHeight="1">
       <c r="A119" s="14" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B119" s="19">
         <v>22.58</v>
@@ -14848,7 +14851,7 @@
     </row>
     <row r="120" ht="15.0" customHeight="1">
       <c r="A120" s="14" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B120" s="18"/>
       <c r="C120" s="18"/>
@@ -14877,7 +14880,7 @@
     </row>
     <row r="121" ht="15.0" customHeight="1">
       <c r="A121" s="14" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B121" s="18"/>
       <c r="C121" s="18"/>
@@ -14924,7 +14927,7 @@
     </row>
     <row r="122" ht="15.0" customHeight="1">
       <c r="A122" s="14" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B122" s="18"/>
       <c r="C122" s="18">
@@ -14979,7 +14982,7 @@
     </row>
     <row r="123" ht="15.0" customHeight="1">
       <c r="A123" s="14" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B123" s="18"/>
       <c r="C123" s="18">
@@ -15026,7 +15029,7 @@
     </row>
     <row r="124" ht="15.0" customHeight="1">
       <c r="A124" s="14" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B124" s="18"/>
       <c r="C124" s="18">
@@ -15073,7 +15076,7 @@
     </row>
     <row r="125" ht="15.0" customHeight="1">
       <c r="A125" s="14" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B125" s="18"/>
       <c r="C125" s="18">
@@ -15126,7 +15129,7 @@
     </row>
     <row r="126" ht="15.0" customHeight="1">
       <c r="A126" s="14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B126" s="18"/>
       <c r="C126" s="15">
@@ -15179,7 +15182,7 @@
     </row>
     <row r="127" ht="15.0" customHeight="1">
       <c r="A127" s="14" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B127" s="18"/>
       <c r="C127" s="18"/>
@@ -15224,7 +15227,7 @@
     </row>
     <row r="128" ht="15.0" customHeight="1">
       <c r="A128" s="14" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B128" s="18"/>
       <c r="C128" s="18"/>
@@ -15253,7 +15256,7 @@
     </row>
     <row r="129" ht="15.0" customHeight="1">
       <c r="A129" s="14" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B129" s="18"/>
       <c r="C129" s="18"/>
@@ -15288,7 +15291,7 @@
     </row>
     <row r="130" ht="15.0" customHeight="1">
       <c r="A130" s="14" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B130" s="18"/>
       <c r="C130" s="15">
@@ -15337,7 +15340,7 @@
     </row>
     <row r="131" ht="15.0" customHeight="1">
       <c r="A131" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B131" s="18"/>
       <c r="C131" s="19">
@@ -15378,7 +15381,7 @@
     </row>
     <row r="132" ht="15.0" customHeight="1">
       <c r="A132" s="14" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B132" s="18"/>
       <c r="C132" s="19">
@@ -15419,7 +15422,7 @@
     </row>
     <row r="133" ht="15.0" customHeight="1">
       <c r="A133" s="14" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B133" s="18"/>
       <c r="C133" s="19">
@@ -15460,7 +15463,7 @@
     </row>
     <row r="134" ht="15.0" customHeight="1">
       <c r="A134" s="14" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B134" s="18"/>
       <c r="C134" s="19">
@@ -15499,7 +15502,7 @@
     </row>
     <row r="135" ht="15.0" customHeight="1">
       <c r="A135" s="14" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B135" s="19">
         <v>0.92</v>
@@ -15570,7 +15573,7 @@
     </row>
     <row r="136" ht="15.0" customHeight="1">
       <c r="A136" s="14" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B136" s="19">
         <v>20.83</v>
@@ -15641,7 +15644,7 @@
     </row>
     <row r="137" ht="15.0" customHeight="1">
       <c r="A137" s="14" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B137" s="19">
         <v>20.83</v>
@@ -15712,7 +15715,7 @@
     </row>
     <row r="138" ht="15.0" customHeight="1">
       <c r="A138" s="14" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B138" s="19">
         <v>1.75</v>
@@ -15783,7 +15786,7 @@
     </row>
     <row r="139" ht="15.0" customHeight="1">
       <c r="A139" s="14" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B139" s="19">
         <v>1.75</v>
@@ -15854,7 +15857,7 @@
     </row>
     <row r="140" ht="15.0" customHeight="1">
       <c r="A140" s="14" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B140" s="19">
         <v>0.08</v>
@@ -16805,7 +16808,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -17191,70 +17194,70 @@
         <v>44</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="R15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="T15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="V15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="W15" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="16" ht="15.0" customHeight="1" outlineLevel="1">
@@ -17330,7 +17333,7 @@
     </row>
     <row r="18">
       <c r="A18" s="12" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -17428,7 +17431,7 @@
     </row>
     <row r="20" ht="15.0" customHeight="1">
       <c r="A20" s="14" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B20" s="18"/>
       <c r="C20" s="18"/>
@@ -17457,7 +17460,7 @@
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="14" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B21" s="18"/>
       <c r="C21" s="18"/>
@@ -17488,7 +17491,7 @@
     </row>
     <row r="22" ht="15.0" customHeight="1">
       <c r="A22" s="14" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B22" s="15">
         <v>557.23</v>
@@ -17517,7 +17520,7 @@
     </row>
     <row r="23" ht="15.0" customHeight="1">
       <c r="A23" s="14" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B23" s="18"/>
       <c r="C23" s="15">
@@ -17570,7 +17573,7 @@
     </row>
     <row r="24" ht="15.0" customHeight="1">
       <c r="A24" s="14" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B24" s="18"/>
       <c r="C24" s="15">
@@ -17639,7 +17642,7 @@
     </row>
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="14" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="15">
@@ -17692,7 +17695,7 @@
     </row>
     <row r="26" ht="15.0" customHeight="1">
       <c r="A26" s="14" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B26" s="18"/>
       <c r="C26" s="19">
@@ -17759,7 +17762,7 @@
     </row>
     <row r="27" ht="15.0" customHeight="1">
       <c r="A27" s="14" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B27" s="18"/>
       <c r="C27" s="18"/>
@@ -17867,7 +17870,7 @@
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="14" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B29" s="18"/>
       <c r="C29" s="15">
@@ -17900,7 +17903,7 @@
     </row>
     <row r="30" ht="15.0" customHeight="1">
       <c r="A30" s="14" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B30" s="18"/>
       <c r="C30" s="19">
@@ -17931,7 +17934,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="14" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B31" s="18"/>
       <c r="C31" s="18">
@@ -17964,7 +17967,7 @@
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="14" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B32" s="18"/>
       <c r="C32" s="22">
@@ -17997,7 +18000,7 @@
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="14" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B33" s="18"/>
       <c r="C33" s="19">
@@ -18030,7 +18033,7 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="14" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B34" s="18"/>
       <c r="C34" s="18">
@@ -18096,7 +18099,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="14" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B36" s="18"/>
       <c r="C36" s="22">
@@ -18161,7 +18164,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="14" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B37" s="18"/>
       <c r="C37" s="19">
@@ -18228,7 +18231,7 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="14" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B38" s="22">
         <v>-17.26</v>
@@ -18299,7 +18302,7 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="14" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B39" s="25">
         <v>-208.66</v>
@@ -18328,7 +18331,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="14" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B40" s="18"/>
       <c r="C40" s="18"/>
@@ -18379,7 +18382,7 @@
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="14" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B41" s="18"/>
       <c r="C41" s="18"/>
@@ -18420,7 +18423,7 @@
     </row>
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="14" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B42" s="18"/>
       <c r="C42" s="19">
@@ -18489,7 +18492,7 @@
     </row>
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="14" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B43" s="18"/>
       <c r="C43" s="18"/>
@@ -18554,7 +18557,7 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="14" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B44" s="18"/>
       <c r="C44" s="19">
@@ -18623,7 +18626,7 @@
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="14" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B45" s="18"/>
       <c r="C45" s="18"/>
@@ -18652,7 +18655,7 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="14" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B46" s="18"/>
       <c r="C46" s="18"/>
@@ -18689,7 +18692,7 @@
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="14" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B47" s="18"/>
       <c r="C47" s="18"/>
@@ -18718,7 +18721,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="16" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B48" s="17">
         <v>331.31</v>
@@ -18789,7 +18792,7 @@
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="14" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B49" s="18"/>
       <c r="C49" s="18"/>
@@ -18818,7 +18821,7 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="14" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B50" s="18"/>
       <c r="C50" s="22">
@@ -18887,7 +18890,7 @@
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="14" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B51" s="18"/>
       <c r="C51" s="22">
@@ -18956,7 +18959,7 @@
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="14" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B52" s="18"/>
       <c r="C52" s="22">
@@ -19015,7 +19018,7 @@
     </row>
     <row r="53" ht="15.0" customHeight="1">
       <c r="A53" s="14" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B53" s="18"/>
       <c r="C53" s="18"/>
@@ -19058,7 +19061,7 @@
     </row>
     <row r="54" ht="15.0" customHeight="1">
       <c r="A54" s="14" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B54" s="18"/>
       <c r="C54" s="18"/>
@@ -19101,7 +19104,7 @@
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="14" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B55" s="18"/>
       <c r="C55" s="18"/>
@@ -19150,7 +19153,7 @@
     </row>
     <row r="56" ht="15.0" customHeight="1">
       <c r="A56" s="14" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B56" s="18"/>
       <c r="C56" s="19">
@@ -19199,7 +19202,7 @@
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="14" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B57" s="18"/>
       <c r="C57" s="18"/>
@@ -19232,7 +19235,7 @@
     </row>
     <row r="58" ht="15.0" customHeight="1">
       <c r="A58" s="14" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B58" s="18"/>
       <c r="C58" s="18"/>
@@ -19263,7 +19266,7 @@
     </row>
     <row r="59" ht="15.0" customHeight="1">
       <c r="A59" s="16" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B59" s="27">
         <v>-149.66</v>
@@ -19334,7 +19337,7 @@
     </row>
     <row r="60" ht="15.0" customHeight="1">
       <c r="A60" s="14" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B60" s="18"/>
       <c r="C60" s="19">
@@ -19395,7 +19398,7 @@
     </row>
     <row r="61" ht="15.0" customHeight="1">
       <c r="A61" s="14" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B61" s="18"/>
       <c r="C61" s="18"/>
@@ -19426,7 +19429,7 @@
     </row>
     <row r="62" ht="15.0" customHeight="1">
       <c r="A62" s="14" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B62" s="18"/>
       <c r="C62" s="22">
@@ -19465,7 +19468,7 @@
     </row>
     <row r="63" ht="15.0" customHeight="1">
       <c r="A63" s="14" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B63" s="18"/>
       <c r="C63" s="18"/>
@@ -19522,7 +19525,7 @@
     </row>
     <row r="64" ht="15.0" customHeight="1">
       <c r="A64" s="14" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B64" s="18"/>
       <c r="C64" s="25">
@@ -19591,7 +19594,7 @@
     </row>
     <row r="65" ht="15.0" customHeight="1">
       <c r="A65" s="14" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B65" s="18"/>
       <c r="C65" s="18"/>
@@ -19622,7 +19625,7 @@
     </row>
     <row r="66" ht="15.0" customHeight="1">
       <c r="A66" s="14" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B66" s="18"/>
       <c r="C66" s="18"/>
@@ -19665,7 +19668,7 @@
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="14" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B67" s="18"/>
       <c r="C67" s="18"/>
@@ -19696,7 +19699,7 @@
     </row>
     <row r="68" ht="15.0" customHeight="1">
       <c r="A68" s="14" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B68" s="18"/>
       <c r="C68" s="25">
@@ -19735,7 +19738,7 @@
     </row>
     <row r="69" ht="15.0" customHeight="1">
       <c r="A69" s="14" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B69" s="18"/>
       <c r="C69" s="22">
@@ -19768,7 +19771,7 @@
     </row>
     <row r="70" ht="15.0" customHeight="1">
       <c r="A70" s="14" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B70" s="18"/>
       <c r="C70" s="18">
@@ -19799,7 +19802,7 @@
     </row>
     <row r="71" ht="15.0" customHeight="1">
       <c r="A71" s="16" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B71" s="27">
         <v>-209.61</v>
@@ -19870,7 +19873,7 @@
     </row>
     <row r="72" ht="15.0" customHeight="1">
       <c r="A72" s="14" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B72" s="22">
         <v>-3.28</v>
@@ -19929,7 +19932,7 @@
     </row>
     <row r="73" ht="15.0" customHeight="1">
       <c r="A73" s="14" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B73" s="19">
         <v>75.01</v>
@@ -20000,7 +20003,7 @@
     </row>
     <row r="74" ht="15.0" customHeight="1">
       <c r="A74" s="14" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B74" s="19">
         <v>42.75</v>
@@ -20071,7 +20074,7 @@
     </row>
     <row r="75" ht="15.0" customHeight="1">
       <c r="A75" s="14" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B75" s="22">
         <v>-27.96</v>
@@ -20126,7 +20129,7 @@
     </row>
     <row r="76" ht="15.0" customHeight="1">
       <c r="A76" s="16" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B76" s="23">
         <v>-31.25</v>
@@ -21141,7 +21144,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -21306,7 +21309,7 @@
         <v>39</v>
       </c>
       <c r="W11" s="7" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="12" ht="15.0" customHeight="1" outlineLevel="1">
@@ -21666,7 +21669,7 @@
     </row>
     <row r="18">
       <c r="A18" s="12" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -21759,12 +21762,12 @@
         <v>70</v>
       </c>
       <c r="W19" s="13" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="20" ht="15.0" customHeight="1">
       <c r="A20" s="28" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B20" s="29"/>
       <c r="C20" s="29"/>
@@ -21791,7 +21794,7 @@
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="30" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B21" s="31">
         <v>3836.39</v>
@@ -21862,7 +21865,7 @@
     </row>
     <row r="22" ht="15.0" customHeight="1">
       <c r="A22" s="30" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B22" s="31">
         <v>3476.55</v>
@@ -21925,7 +21928,7 @@
     </row>
     <row r="23" ht="15.0" customHeight="1">
       <c r="A23" s="28" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B23" s="29"/>
       <c r="C23" s="29"/>
@@ -21952,7 +21955,7 @@
     </row>
     <row r="24" ht="15.0" customHeight="1">
       <c r="A24" s="30" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B24" s="31">
         <v>3222.82</v>
@@ -22023,7 +22026,7 @@
     </row>
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="30" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B25" s="31">
         <v>3053.98</v>
@@ -22086,7 +22089,7 @@
     </row>
     <row r="26" ht="15.0" customHeight="1">
       <c r="A26" s="28" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B26" s="29"/>
       <c r="C26" s="29"/>
@@ -22113,7 +22116,7 @@
     </row>
     <row r="27" ht="15.0" customHeight="1">
       <c r="A27" s="30" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B27" s="31">
         <v>145.78</v>
@@ -22184,7 +22187,7 @@
     </row>
     <row r="28" ht="15.0" customHeight="1">
       <c r="A28" s="30" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B28" s="31">
         <v>147.45</v>
@@ -22247,7 +22250,7 @@
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="28" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B29" s="29"/>
       <c r="C29" s="29"/>
@@ -22274,7 +22277,7 @@
     </row>
     <row r="30" ht="15.0" customHeight="1">
       <c r="A30" s="30" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B30" s="34">
         <v>11.79</v>
@@ -22345,7 +22348,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="30" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B31" s="34">
         <v>8.58</v>
@@ -22408,7 +22411,7 @@
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="28" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B32" s="29"/>
       <c r="C32" s="29"/>
@@ -22435,7 +22438,7 @@
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="30" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B33" s="34">
         <v>2.22</v>
@@ -22506,7 +22509,7 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="30" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B34" s="34">
         <v>1.66</v>
@@ -22569,7 +22572,7 @@
     </row>
     <row r="35" ht="15.0" customHeight="1">
       <c r="A35" s="30" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B35" s="34">
         <v>3.17</v>
@@ -22640,7 +22643,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="30" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B36" s="34">
         <v>2.37</v>
@@ -22703,7 +22706,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="28" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B37" s="29"/>
       <c r="C37" s="29"/>
@@ -22730,7 +22733,7 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="30" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B38" s="33">
         <v>1.62</v>
@@ -22801,7 +22804,7 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="30" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B39" s="33">
         <v>1.98</v>
@@ -22864,7 +22867,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="28" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B40" s="29"/>
       <c r="C40" s="29"/>
@@ -22891,7 +22894,7 @@
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="30" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B41" s="32"/>
       <c r="C41" s="32"/>
@@ -22956,7 +22959,7 @@
     </row>
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="30" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B42" s="33">
         <v>45.73</v>
@@ -23019,7 +23022,7 @@
     </row>
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="28" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B43" s="29"/>
       <c r="C43" s="29"/>
@@ -23046,7 +23049,7 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="30" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B44" s="33">
         <v>0.71</v>
@@ -23117,7 +23120,7 @@
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="30" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B45" s="33">
         <v>0.88</v>
@@ -23180,7 +23183,7 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="28" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B46" s="29"/>
       <c r="C46" s="29"/>
@@ -23207,7 +23210,7 @@
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="30" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B47" s="33">
         <v>8.48</v>
@@ -23274,7 +23277,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="30" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B48" s="33">
         <v>11.65</v>
@@ -23337,7 +23340,7 @@
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="28" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B49" s="29"/>
       <c r="C49" s="29"/>
@@ -23364,7 +23367,7 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="30" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B50" s="33">
         <v>7.22</v>
@@ -23435,7 +23438,7 @@
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="30" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B51" s="33">
         <v>9.25</v>
@@ -23498,7 +23501,7 @@
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="28" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B52" s="29"/>
       <c r="C52" s="29"/>
@@ -23525,7 +23528,7 @@
     </row>
     <row r="53" ht="15.0" customHeight="1">
       <c r="A53" s="30" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B53" s="33">
         <v>14.13</v>
@@ -23596,7 +23599,7 @@
     </row>
     <row r="54" ht="15.0" customHeight="1">
       <c r="A54" s="30" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B54" s="33">
         <v>20.48</v>
@@ -23659,7 +23662,7 @@
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="28" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B55" s="29"/>
       <c r="C55" s="29"/>
@@ -23686,7 +23689,7 @@
     </row>
     <row r="56" ht="15.0" customHeight="1">
       <c r="A56" s="30" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B56" s="33">
         <v>14.6</v>
@@ -23757,7 +23760,7 @@
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="30" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B57" s="33">
         <v>1.98</v>
@@ -23820,7 +23823,7 @@
     </row>
     <row r="58" ht="15.0" customHeight="1">
       <c r="A58" s="28" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B58" s="29"/>
       <c r="C58" s="29"/>
@@ -23847,7 +23850,7 @@
     </row>
     <row r="59" ht="15.0" customHeight="1">
       <c r="A59" s="30" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B59" s="33">
         <v>0.68</v>
@@ -23916,7 +23919,7 @@
     </row>
     <row r="60" ht="15.0" customHeight="1">
       <c r="A60" s="30" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B60" s="33">
         <v>0.75</v>
@@ -23977,7 +23980,7 @@
     </row>
     <row r="61" ht="15.0" customHeight="1">
       <c r="A61" s="28" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B61" s="29"/>
       <c r="C61" s="29"/>
@@ -24004,7 +24007,7 @@
     </row>
     <row r="62" ht="15.0" customHeight="1">
       <c r="A62" s="30" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B62" s="33">
         <v>0.84</v>
@@ -24075,7 +24078,7 @@
     </row>
     <row r="63" ht="15.0" customHeight="1">
       <c r="A63" s="30" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B63" s="33">
         <v>0.98</v>
@@ -24138,7 +24141,7 @@
     </row>
     <row r="64" ht="15.0" customHeight="1">
       <c r="A64" s="28" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B64" s="29"/>
       <c r="C64" s="29"/>
@@ -24165,7 +24168,7 @@
     </row>
     <row r="65" ht="15.0" customHeight="1">
       <c r="A65" s="30" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B65" s="33">
         <v>7.44</v>
@@ -24236,7 +24239,7 @@
     </row>
     <row r="66" ht="15.0" customHeight="1">
       <c r="A66" s="30" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B66" s="33">
         <v>8.48</v>
@@ -24299,7 +24302,7 @@
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="28" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B67" s="29"/>
       <c r="C67" s="29"/>
@@ -24326,7 +24329,7 @@
     </row>
     <row r="68" ht="15.0" customHeight="1">
       <c r="A68" s="30" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B68" s="33">
         <v>9.15</v>
@@ -24395,7 +24398,7 @@
     </row>
     <row r="69" ht="15.0" customHeight="1">
       <c r="A69" s="30" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B69" s="33">
         <v>11.66</v>
@@ -24458,7 +24461,7 @@
     </row>
     <row r="70" ht="15.0" customHeight="1">
       <c r="A70" s="28" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B70" s="29"/>
       <c r="C70" s="29"/>
@@ -24485,7 +24488,7 @@
     </row>
     <row r="71" ht="15.0" customHeight="1">
       <c r="A71" s="30" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B71" s="33">
         <v>10.09</v>
@@ -24552,7 +24555,7 @@
     </row>
     <row r="72" ht="15.0" customHeight="1">
       <c r="A72" s="30" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B72" s="33">
         <v>13.06</v>

</xml_diff>